<commit_message>
feat: Gemini 3단계 분류 구현
- 3단계 폭포식 가맹점 분류 (소상공인DB -> SBERT -> Gemini fallback)
- 세부 품목명 분류 (FAST_TRACK_MAP -> SBERT -> Gemini fallback)
- 미분류 Safe-Default 반환 (대분류 평균 탄소계수 사용)
- EXIOBASE 기반 탄소배출량 계산 및 carbon.py 구현
- 영수증 분류 결과 DB 저장 및 기간별 통계 자동 집계 (record_service.py)
- FastAPI Depends 패턴 DB 연결 공유
- SBERT 카테고리 임베딩 prefix 불일치 수정 (bare text 통일)
- 카셰어링/렌터카 분류 키워드 추가 (MERCHANT_KEYWORD_MAP)
- scripts 파일명 snake_case 규칙으로 정리 및 data_prep 서브패키지 분리
</commit_message>
<xml_diff>
--- a/data/category_carbon_v2.xlsx
+++ b/data/category_carbon_v2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcbri\OneDrive\바탕 화면\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcbri\PycharmProjects\GreenStep\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F0C4608-04A5-4B1A-85DF-712226370C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC5C347E-5677-4861-A082-E34DC893033C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0F6C9620-84A5-47F2-85DD-B3E6F7730BB0}"/>
   </bookViews>
@@ -20,22 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="89">
   <si>
     <t xml:space="preserve">메인 카테고리 </t>
   </si>
@@ -82,18 +72,6 @@
     <t>교통</t>
   </si>
   <si>
-    <t>LPG</t>
-  </si>
-  <si>
-    <t>경유</t>
-  </si>
-  <si>
-    <t>휘발유</t>
-  </si>
-  <si>
-    <t>전기차</t>
-  </si>
-  <si>
     <t>대중교통</t>
   </si>
   <si>
@@ -241,9 +219,6 @@
     <t>무알콜음료</t>
   </si>
   <si>
-    <t>알코올 음료</t>
-  </si>
-  <si>
     <t>빵</t>
   </si>
   <si>
@@ -293,13 +268,45 @@
   </si>
   <si>
     <t>구분하지 못하는 것</t>
+  </si>
+  <si>
+    <t>자동차구입</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>교통</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>자동차정비</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>알코올음료</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>경유충전</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LPG충전</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>휘발유충전</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>전기차충전</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -314,6 +321,12 @@
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0A0A0A"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -338,11 +351,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -659,7 +675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D01474DA-6137-4A88-9E69-40BEBEAA13F3}">
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="21.19921875" customWidth="1"/>
@@ -767,7 +783,7 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>86</v>
       </c>
       <c r="C9">
         <v>2.849E-3</v>
@@ -778,7 +794,7 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>85</v>
       </c>
       <c r="C10">
         <v>1.316843E-3</v>
@@ -789,7 +805,7 @@
         <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>87</v>
       </c>
       <c r="C11">
         <v>1.1250030000000001E-3</v>
@@ -800,7 +816,7 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>88</v>
       </c>
       <c r="C12">
         <v>1.1525999999999999E-3</v>
@@ -808,688 +824,711 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>82</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="1">
-        <v>5.1858299999999998E-5</v>
+        <v>81</v>
+      </c>
+      <c r="C13" s="2">
+        <v>1.5523100000000001E-3</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>82</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14" s="1">
-        <v>2.9560700000000001E-7</v>
+        <v>83</v>
+      </c>
+      <c r="C14" s="2">
+        <v>1.2313100000000001E-4</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15">
-        <v>1.43545E-4</v>
+        <v>16</v>
+      </c>
+      <c r="C15" s="1">
+        <v>5.1858299999999998E-5</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16">
-        <v>1.3899999999999999E-4</v>
+        <v>17</v>
+      </c>
+      <c r="C16" s="1">
+        <v>2.9560700000000001E-7</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C17">
-        <v>4.6548999999999999E-4</v>
+        <v>1.43545E-4</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C18">
-        <v>1.8830999999999999E-4</v>
+        <v>1.3899999999999999E-4</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C19">
-        <v>2.42477E-4</v>
+        <v>4.6548999999999999E-4</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C20">
-        <v>2.3713E-4</v>
+        <v>1.8830999999999999E-4</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C21">
-        <v>1.5415000000000001E-4</v>
+        <v>2.42477E-4</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C22">
-        <v>2.1644490000000001E-3</v>
+        <v>2.3713E-4</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C23">
-        <v>1.8150999999999999E-4</v>
+        <v>1.5415000000000001E-4</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C24">
-        <v>3.6999999999999998E-5</v>
+        <v>2.1644490000000001E-3</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C25">
-        <v>1.6750000000000001E-4</v>
+        <v>1.8150999999999999E-4</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
         <v>29</v>
       </c>
-      <c r="B26" t="s">
-        <v>35</v>
-      </c>
       <c r="C26">
-        <v>4.7367999999999998E-4</v>
+        <v>3.6999999999999998E-5</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C27">
-        <v>6.6000000000000005E-5</v>
+        <v>1.6750000000000001E-4</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C28">
-        <v>8.9099999999999997E-5</v>
+        <v>4.7367999999999998E-4</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="B29" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C29">
-        <v>2.6403E-4</v>
+        <v>6.6000000000000005E-5</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="B30" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C30">
-        <v>4.057E-4</v>
+        <v>8.9099999999999997E-5</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B31" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C31">
-        <v>1.1325E-4</v>
+        <v>2.6403E-4</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C32">
-        <v>3.0180000000000002E-4</v>
+        <v>4.057E-4</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B33" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C33">
-        <v>4.2185999999999998E-4</v>
+        <v>1.1325E-4</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" t="s">
         <v>38</v>
       </c>
-      <c r="B34" t="s">
-        <v>44</v>
-      </c>
       <c r="C34">
-        <v>1.5634000000000001E-4</v>
+        <v>3.0180000000000002E-4</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C35">
-        <v>1.0906E-4</v>
+        <v>4.2185999999999998E-4</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C36">
-        <v>1.7741E-4</v>
+        <v>1.5634000000000001E-4</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B37" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C37">
-        <v>7.6719999999999997E-5</v>
+        <v>1.0906E-4</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C38">
-        <v>1.4584E-4</v>
+        <v>1.7741E-4</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B39" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C39">
-        <v>2.1641999999999999E-4</v>
+        <v>7.6719999999999997E-5</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B40" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C40">
-        <v>2.8778000000000001E-4</v>
+        <v>1.4584E-4</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B41" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C41">
-        <v>2.1458999999999999E-4</v>
+        <v>2.1641999999999999E-4</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B42" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C42">
-        <v>2.9749000000000003E-4</v>
+        <v>2.8778000000000001E-4</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A43" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B43" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C43">
-        <v>2.3188000000000001E-4</v>
+        <v>2.1458999999999999E-4</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B44" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C44">
-        <v>7.1740000000000001E-5</v>
+        <v>2.9749000000000003E-4</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B45" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C45">
-        <v>9.8880000000000002E-5</v>
+        <v>2.3188000000000001E-4</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A46" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B46" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C46">
-        <v>1.3993999999999999E-4</v>
+        <v>7.1740000000000001E-5</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A47" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B47" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C47">
-        <v>1.6992999999999999E-4</v>
+        <v>9.8880000000000002E-5</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B48" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C48">
-        <v>1.9523000000000001E-4</v>
+        <v>1.3993999999999999E-4</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A49" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B49" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C49">
-        <v>3.4260000000000001E-5</v>
+        <v>1.6992999999999999E-4</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A50" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B50" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C50">
-        <v>9.4469999999999995E-5</v>
+        <v>1.9523000000000001E-4</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A51" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B51" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C51">
-        <v>7.9870000000000006E-5</v>
+        <v>3.4260000000000001E-5</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A52" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B52" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C52">
-        <v>4.2034E-4</v>
+        <v>9.4469999999999995E-5</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B53" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C53">
-        <v>1.4292999999999999E-4</v>
+        <v>7.9870000000000006E-5</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A54" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B54" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C54">
-        <v>1.8310000000000001E-4</v>
+        <v>4.2034E-4</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A55" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B55" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C55">
-        <v>1.2370999999999999E-4</v>
+        <v>1.4292999999999999E-4</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A56" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B56" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C56">
-        <v>1.4839000000000001E-4</v>
+        <v>1.8310000000000001E-4</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A57" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B57" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C57">
-        <v>1.6006000000000001E-4</v>
+        <v>1.2370999999999999E-4</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A58" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B58" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C58">
-        <v>4.2599999999999999E-5</v>
+        <v>1.4839000000000001E-4</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A59" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B59" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C59">
-        <v>2.7608E-4</v>
+        <v>1.6006000000000001E-4</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A60" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B60" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="C60">
-        <v>3.4262000000000002E-4</v>
+        <v>4.2599999999999999E-5</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A61" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B61" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C61">
-        <v>1.0378999999999999E-4</v>
+        <v>2.7608E-4</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A62" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B62" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C62">
-        <v>8.6840000000000002E-5</v>
+        <v>3.4262000000000002E-4</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A63" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B63" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C63">
-        <v>4.7663000000000002E-4</v>
+        <v>1.0378999999999999E-4</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A64" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B64" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C64">
-        <v>8.9679999999999995E-5</v>
+        <v>8.6840000000000002E-5</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A65" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B65" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C65">
-        <v>1.2488000000000001E-4</v>
+        <v>4.7663000000000002E-4</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A66" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B66" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C66">
-        <v>1.0665E-4</v>
+        <v>8.9679999999999995E-5</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A67" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B67" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="C67">
-        <v>1.5142000000000001E-4</v>
+        <v>1.2488000000000001E-4</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A68" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B68" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="C68">
-        <v>1.9165E-4</v>
+        <v>1.0665E-4</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A69" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B69" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="C69">
-        <v>5.6390000000000001E-5</v>
+        <v>1.5142000000000001E-4</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A70" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B70" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="C70">
-        <v>1.1496E-4</v>
+        <v>1.9165E-4</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A71" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B71" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C71">
-        <v>8.4740000000000005E-5</v>
+        <v>5.6390000000000001E-5</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A72" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B72" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="C72">
-        <v>6.4460000000000003E-5</v>
+        <v>1.1496E-4</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A73" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B73" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="C73">
-        <v>8.6609999999999999E-5</v>
+        <v>8.4740000000000005E-5</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A74" t="s">
-        <v>84</v>
+        <v>34</v>
       </c>
       <c r="B74" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="C74">
+        <v>6.4460000000000003E-5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A75" t="s">
+        <v>34</v>
+      </c>
+      <c r="B75" t="s">
+        <v>78</v>
+      </c>
+      <c r="C75">
+        <v>8.6609999999999999E-5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A76" t="s">
+        <v>79</v>
+      </c>
+      <c r="B76" t="s">
+        <v>80</v>
+      </c>
+      <c r="C76">
         <v>1E-8</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>